<commit_message>
feat: add bulk import Excel templates for categories, tests, packages, laboratories, and master records
</commit_message>
<xml_diff>
--- a/public/templates/2_Litmus_Tests_Bulk_Template.xlsx
+++ b/public/templates/2_Litmus_Tests_Bulk_Template.xlsx
@@ -488,24 +488,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:Q7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="148" customWidth="1" min="1" max="1"/>
-    <col width="101" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="41" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="25" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="41" customWidth="1" min="8" max="8"/>
+    <col width="101" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="121" customWidth="1" min="14" max="14"/>
-    <col width="94" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
+    <col width="25" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="121" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -523,70 +525,80 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>discountType</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>discountValue</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>offerPrice</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>turnAroundTime</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>testType</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>fssaiMethod</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
           <t>description</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>imageUrl</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>fssaiMethod</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>testType</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>turnAroundTime</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>creatorType</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>labName</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>isApplicableToAll</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>applicableCategories</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>applicableSubcategories</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>isPopular</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>discountType</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>discountValue</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>parameters</t>
         </is>
@@ -598,9 +610,9 @@
           <t>REQUIRED *</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>REQUIRED *</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -663,9 +675,19 @@
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr">
-        <is>
-          <t>REQUIRED *</t>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="P3" s="4" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="Q3" s="4" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
         </is>
       </c>
     </row>
@@ -675,66 +697,72 @@
           <t>Milk Fat &amp; Solids Analysis</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="5" t="n">
+        <v>400</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>PERCENTAGE</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>360</v>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>24 Hours</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Chemical</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>IS:1479 (Part I) - 1960</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>Complete determination of milk fat by Gerber method and solids-not-fat (SNF) calculation.</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>https://example.com/icons/milk-fat.png</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>IS:1479 (Part I) - 1960</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>Chemical</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>24 Hours</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>ADMIN</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr"/>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="L4" s="5" t="inlineStr"/>
+      <c r="M4" s="5" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>Dairy &amp; Milk Products</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="O4" s="5" t="inlineStr">
         <is>
           <t>Raw Milk, Pasteurized Milk</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="P4" s="5" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
-        <is>
-          <t>PERCENTAGE</t>
-        </is>
-      </c>
-      <c r="N4" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="Q4" s="5" t="inlineStr">
         <is>
           <t>Total Fat:%:3.0:8.0:180; Solids Not Fat (SNF):%:8.0:10.5:120; Density:g/ml:1.026:1.032:100</t>
         </is>
@@ -746,62 +774,68 @@
           <t>Cheese &amp; Paneer Moisture &amp; Fat Panel</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="5" t="n">
+        <v>550</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>550</v>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>24 Hours</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Chemical</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>IS:2785 - 1979 / FSSAI Manual 01</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>Determination of moisture and fat on dry basis for cheese, paneer, and cottage cheese.</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>IS:2785 - 1979 / FSSAI Manual 01</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Chemical</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>24 Hours</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr"/>
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>ADMIN</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr"/>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="L5" s="5" t="inlineStr"/>
+      <c r="M5" s="5" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="N5" s="5" t="inlineStr">
         <is>
           <t>Dairy &amp; Milk Products</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="O5" s="5" t="inlineStr">
         <is>
           <t>Cheese &amp; Paneer</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr">
+      <c r="P5" s="5" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="M5" s="5" t="inlineStr">
-        <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="N5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" s="5" t="inlineStr">
+      <c r="Q5" s="5" t="inlineStr">
         <is>
           <t>Moisture Content:%:0:60.0:250; Fat on Dry Basis:%:45.0:70.0:300</t>
         </is>
@@ -813,54 +847,60 @@
           <t>Microbial Safety Screen (E. Coli &amp; Coliforms)</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="5" t="n">
+        <v>800</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>800</v>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>48 Hours</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Microbiology</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>IS:5401 (Part 1):2012 / ISO 4832:2006</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>Quantitative enumeration of total viable coliforms and Escherichia coli in food &amp; water matrices.</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>IS:5401 (Part 1):2012 / ISO 4832:2006</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Microbiology</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>48 Hours</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr"/>
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>ADMIN</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr"/>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="L6" s="5" t="inlineStr"/>
+      <c r="M6" s="5" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr"/>
-      <c r="K6" s="5" t="inlineStr"/>
-      <c r="L6" s="5" t="inlineStr">
+      <c r="N6" s="5" t="inlineStr"/>
+      <c r="O6" s="5" t="inlineStr"/>
+      <c r="P6" s="5" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="M6" s="5" t="inlineStr">
-        <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="N6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" s="5" t="inlineStr">
+      <c r="Q6" s="5" t="inlineStr">
         <is>
           <t>Total Coliform Count:cfu/g:0:10:350; E. Coli Count:cfu/g:0:0:450</t>
         </is>
@@ -872,53 +912,60 @@
           <t>Heavy Metals Residue Panel</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="5" t="n">
+        <v>1750</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>200</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>1550</v>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>72 Hours</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Chemical</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>AOAC 2015.01 / FSSAI Manual 02</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>Inductively Coupled Plasma Mass Spectrometry (ICP-MS) detection for toxic heavy metals.</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>AOAC 2015.01 / FSSAI Manual 02</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Chemical</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>72 Hours</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>ADMIN</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr"/>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr"/>
       <c r="K7" s="5" t="inlineStr">
         <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr"/>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N7" s="5" t="inlineStr"/>
+      <c r="O7" s="5" t="inlineStr"/>
+      <c r="P7" s="5" t="inlineStr">
+        <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="L7" s="5" t="inlineStr">
-        <is>
-          <t>FLAT</t>
-        </is>
-      </c>
-      <c r="M7" s="5" t="n">
-        <v>200</v>
-      </c>
-      <c r="N7" s="5" t="inlineStr">
+      <c r="Q7" s="5" t="inlineStr">
         <is>
           <t>Lead (Pb):ppm:0.0:0.1:400; Cadmium (Cd):ppm:0.0:0.05:400; Arsenic (As):ppm:0.0:0.1:450; Mercury (Hg):ppm:0.0:0.01:450</t>
         </is>
@@ -926,7 +973,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>